<commit_message>
Finalização do trabalho, parte 1
</commit_message>
<xml_diff>
--- a/Trabalho Final/padaria_RF.xlsx
+++ b/Trabalho Final/padaria_RF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ASIS\Trabalho Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F88026-0123-4C0C-BFDD-7AA3E1D59C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F79CB2-F098-4A43-9FCC-D25D5980733E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="modelo RF" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="108">
   <si>
     <t>Campo</t>
   </si>
@@ -193,9 +193,6 @@
     <t>Exemplos</t>
   </si>
   <si>
-    <t>Exemplo de RNF - Desempenho</t>
-  </si>
-  <si>
     <t>ID do Requisito (RNF)</t>
   </si>
   <si>
@@ -211,13 +208,7 @@
     <t>Requisito</t>
   </si>
   <si>
-    <t>O tempo de resposta do servidor para a página inicial não deve exceder 1.5 segundos.</t>
-  </si>
-  <si>
     <t>Métrica de Teste</t>
-  </si>
-  <si>
-    <t>O teste deve medir o tempo de resposta em 1000 acessos simultâneos.</t>
   </si>
   <si>
     <t>-------------</t>
@@ -226,19 +217,7 @@
     <t>--------------------------------------------------------------------------------</t>
   </si>
   <si>
-    <t>Exemplo de RNF - Segurança</t>
-  </si>
-  <si>
-    <t>RNF-S05</t>
-  </si>
-  <si>
     <t>Segurança</t>
-  </si>
-  <si>
-    <t>Todas as senhas de usuários devem ser armazenadas utilizando o algoritmo de hash SHA-256.</t>
-  </si>
-  <si>
-    <t>Verificar se a coluna do banco de dados usa o padrão de criptografia SHA-256.</t>
   </si>
   <si>
     <t>MODELO REQUISITOS NÃO FUNCIONAIS</t>
@@ -273,12 +252,120 @@
   <si>
     <t>Voltar à página inicial do módulo de produtos no módulo; Ou excluir outro produto</t>
   </si>
+  <si>
+    <t>O teste deve medir o tempo de execução das querys em 10 acessos simultâneos.</t>
+  </si>
+  <si>
+    <t>O tempo de execução das querys no banco de dados não deve exceder 2 segundos.</t>
+  </si>
+  <si>
+    <t>RNF-D02</t>
+  </si>
+  <si>
+    <t>O tempo de abertura e troca entre as telas não deve exceder 2 segundos.</t>
+  </si>
+  <si>
+    <t>O teste deve medir o tempo de abertura ou troca entre as telas com apenas uma instância do sistema aberta, com a máquina em menos de 50% de uso do processador e da memória RAM.</t>
+  </si>
+  <si>
+    <t>RNF-S01</t>
+  </si>
+  <si>
+    <t>Todas as senhas de usuários devem ser armazenadas utilizando o algoritmo de hash SHA-512.</t>
+  </si>
+  <si>
+    <t>Desempenho das querys no Banco de Dados</t>
+  </si>
+  <si>
+    <t>Desempenho das telas do sistema</t>
+  </si>
+  <si>
+    <t>Gestão de Acessos</t>
+  </si>
+  <si>
+    <t>O sistema deve implementar gestão de acessos baseada em fução de cada colaborador, de forma simples e eficiênte.</t>
+  </si>
+  <si>
+    <t>Verificar se o sistema sempre gera o hash, e envia somente o hash ao banco de dados.</t>
+  </si>
+  <si>
+    <t>RNF-S02</t>
+  </si>
+  <si>
+    <t>Verificar se os usuários conseguem acessar somente o necessário, de acordo com a função exercida na empresa.</t>
+  </si>
+  <si>
+    <t>Criptografia de senhas</t>
+  </si>
+  <si>
+    <t>Cumprimento das leis de uso de dados</t>
+  </si>
+  <si>
+    <t>RNF-S03</t>
+  </si>
+  <si>
+    <t>O sistema deve atender às leis e implementar as boas práticas de Proteção de dados, como a LGPD e demais regulatórios de proteção de dados.</t>
+  </si>
+  <si>
+    <t>Expor o sistema a análise de auditoria de segurança e proteção de dados.</t>
+  </si>
+  <si>
+    <t>RNF-A01</t>
+  </si>
+  <si>
+    <t>Agilidade na utilização</t>
+  </si>
+  <si>
+    <t>Acessibilidade</t>
+  </si>
+  <si>
+    <t>O sistema deve realizar todas as ações com a quantinade mínima de clicks e interações possível, para agilizar o atendimento aos clientes.</t>
+  </si>
+  <si>
+    <t>Analisar junto a área de negócio se os passos para a venda estão eficientes e com o número mínimo de interação possível</t>
+  </si>
+  <si>
+    <t>RNF-A02</t>
+  </si>
+  <si>
+    <t>Auto ajuda na utilização</t>
+  </si>
+  <si>
+    <t>O sistema deve conter mensagems de ajuda, simples e objetivas, ao colocar o mouse sobre íconhes de dúvidas.</t>
+  </si>
+  <si>
+    <t>Um usuário que nunca utilizou o sistema, deve conseguir realizar as vendas e gestão de produtos, sem a ajuda constante de outra pessoa.</t>
+  </si>
+  <si>
+    <t>RNF-A03</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir trocar entre os campos nos mecanismos de busca, cadastro, alteração, vendas, usando a tecla "Tab" para passar para o próximo campo, e, as teclas "Shift + Tab" para voltar para o campo anterior.</t>
+  </si>
+  <si>
+    <t>Testar se todos os campos podem ser acessados sem usar o mouse, apenas com os comandos no teclado.</t>
+  </si>
+  <si>
+    <t>Agilidade na troca entre campos</t>
+  </si>
+  <si>
+    <t>Confirmações para ações críticas</t>
+  </si>
+  <si>
+    <t>RNF-A04</t>
+  </si>
+  <si>
+    <t>O sistema deve solicitar a confirmação do usuário, antes de realizar qualquer ação crítica que não pode ser desfeita, como excluir um produto.</t>
+  </si>
+  <si>
+    <t>Testar se nenhuma ação crítica pode ser feita por engano, por falta da confirmação.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -373,6 +460,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -388,7 +490,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -448,11 +550,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -482,14 +608,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -501,8 +626,27 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -946,13 +1090,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1">
-      <c r="A1" s="15" t="s">
-        <v>74</v>
+      <c r="A1" s="14" t="s">
+        <v>67</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="3" spans="1:25" ht="20.25">
       <c r="A3" s="7" t="s">
@@ -1084,7 +1228,7 @@
         <v>16</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="30" customHeight="1">
@@ -1112,7 +1256,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="30" customHeight="1">
@@ -1195,7 +1339,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="31.5">
@@ -1211,7 +1355,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30">
@@ -1219,21 +1363,21 @@
         <v>21</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="12"/>
     </row>
     <row r="27" spans="1:5" ht="23.25">
-      <c r="A27" s="15" t="s">
-        <v>75</v>
+      <c r="A27" s="14" t="s">
+        <v>68</v>
       </c>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="17"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" spans="1:5" ht="12.75">
       <c r="A28" s="10"/>
@@ -1276,13 +1420,13 @@
       <c r="A32" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="13" t="s">
         <v>24</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="E32" s="13" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1378,8 +1522,8 @@
       <c r="D39" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E39" s="18" t="s">
-        <v>76</v>
+      <c r="E39" s="13" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1392,8 +1536,8 @@
       <c r="D40" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E40" s="18" t="s">
-        <v>77</v>
+      <c r="E40" s="13" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="12.75">
@@ -1421,7 +1565,7 @@
       <c r="A44" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B44" s="18" t="s">
+      <c r="B44" s="13" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1461,8 +1605,8 @@
       <c r="A49" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="18" t="s">
-        <v>78</v>
+      <c r="B49" s="13" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="60">
@@ -5204,7 +5348,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Y1002"/>
+  <dimension ref="A1:Y1008"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.42578125" customWidth="1"/>
@@ -5247,7 +5391,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -5275,10 +5419,10 @@
     </row>
     <row r="3" spans="1:25" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -5306,10 +5450,10 @@
     </row>
     <row r="4" spans="1:25" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -5337,10 +5481,10 @@
     </row>
     <row r="5" spans="1:25" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -5368,10 +5512,10 @@
     </row>
     <row r="6" spans="1:25" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -5399,10 +5543,10 @@
     </row>
     <row r="7" spans="1:25" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -5428,12 +5572,12 @@
       <c r="X7" s="3"/>
       <c r="Y7" s="3"/>
     </row>
-    <row r="8" spans="1:25" ht="30" customHeight="1">
+    <row r="8" spans="1:25" ht="23.25" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -5461,10 +5605,10 @@
     </row>
     <row r="9" spans="1:25" ht="30" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -5490,12 +5634,12 @@
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
     </row>
-    <row r="10" spans="1:25" ht="30" customHeight="1">
+    <row r="10" spans="1:25" ht="40.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -5521,12 +5665,12 @@
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
     </row>
-    <row r="11" spans="1:25" ht="30" customHeight="1">
+    <row r="11" spans="1:25" ht="35.25" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -5552,12 +5696,12 @@
       <c r="X11" s="3"/>
       <c r="Y11" s="3"/>
     </row>
-    <row r="12" spans="1:25" ht="30" customHeight="1">
+    <row r="12" spans="1:25" ht="54" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -5583,9 +5727,13 @@
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
     </row>
-    <row r="13" spans="1:25" ht="12.75">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+    <row r="13" spans="1:25" ht="15.75" customHeight="1">
+      <c r="A13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -5610,9 +5758,13 @@
       <c r="X13" s="3"/>
       <c r="Y13" s="3"/>
     </row>
-    <row r="14" spans="1:25" ht="12.75">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+    <row r="14" spans="1:25" ht="30" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>81</v>
+      </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -5637,9 +5789,13 @@
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
     </row>
-    <row r="15" spans="1:25" ht="12.75">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+    <row r="15" spans="1:25" ht="30" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>77</v>
+      </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
@@ -5664,9 +5820,13 @@
       <c r="X15" s="3"/>
       <c r="Y15" s="3"/>
     </row>
-    <row r="16" spans="1:25" ht="12.75">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+    <row r="16" spans="1:25" ht="30" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
@@ -5691,9 +5851,13 @@
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
     </row>
-    <row r="17" spans="1:25" ht="12.75">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+    <row r="17" spans="1:25" ht="37.5" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>82</v>
+      </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -5718,9 +5882,13 @@
       <c r="X17" s="3"/>
       <c r="Y17" s="3"/>
     </row>
-    <row r="18" spans="1:25" ht="12.75">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+    <row r="18" spans="1:25" ht="30" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -5745,9 +5913,13 @@
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
     </row>
-    <row r="19" spans="1:25" ht="12.75">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+    <row r="19" spans="1:25" ht="15">
+      <c r="A19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -5772,9 +5944,13 @@
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
     </row>
-    <row r="20" spans="1:25" ht="12.75">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+    <row r="20" spans="1:25">
+      <c r="A20" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>86</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -5799,9 +5975,13 @@
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
     </row>
-    <row r="21" spans="1:25" ht="12.75">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
+    <row r="21" spans="1:25" ht="47.25">
+      <c r="A21" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
@@ -5826,9 +6006,13 @@
       <c r="X21" s="3"/>
       <c r="Y21" s="3"/>
     </row>
-    <row r="22" spans="1:25" ht="12.75">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
+    <row r="22" spans="1:25">
+      <c r="A22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
@@ -5853,9 +6037,13 @@
       <c r="X22" s="3"/>
       <c r="Y22" s="3"/>
     </row>
-    <row r="23" spans="1:25" ht="12.75">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
+    <row r="23" spans="1:25" ht="30">
+      <c r="A23" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>78</v>
+      </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
@@ -5880,9 +6068,13 @@
       <c r="X23" s="3"/>
       <c r="Y23" s="3"/>
     </row>
-    <row r="24" spans="1:25" ht="12.75">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
+    <row r="24" spans="1:25" ht="31.5">
+      <c r="A24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>83</v>
+      </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
@@ -5907,9 +6099,13 @@
       <c r="X24" s="3"/>
       <c r="Y24" s="3"/>
     </row>
-    <row r="25" spans="1:25" ht="12.75">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
+    <row r="25" spans="1:25" ht="15">
+      <c r="A25" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
@@ -5934,9 +6130,13 @@
       <c r="X25" s="3"/>
       <c r="Y25" s="3"/>
     </row>
-    <row r="26" spans="1:25" ht="12.75">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
+    <row r="26" spans="1:25">
+      <c r="A26" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -5961,9 +6161,13 @@
       <c r="X26" s="3"/>
       <c r="Y26" s="3"/>
     </row>
-    <row r="27" spans="1:25" ht="12.75">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
+    <row r="27" spans="1:25" ht="47.25">
+      <c r="A27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
@@ -5988,9 +6192,13 @@
       <c r="X27" s="3"/>
       <c r="Y27" s="3"/>
     </row>
-    <row r="28" spans="1:25" ht="12.75">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
+    <row r="28" spans="1:25">
+      <c r="A28" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -6015,9 +6223,13 @@
       <c r="X28" s="3"/>
       <c r="Y28" s="3"/>
     </row>
-    <row r="29" spans="1:25" ht="12.75">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
+    <row r="29" spans="1:25" ht="45">
+      <c r="A29" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -6042,9 +6254,13 @@
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
     </row>
-    <row r="30" spans="1:25" ht="12.75">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
+    <row r="30" spans="1:25" ht="31.5">
+      <c r="A30" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
@@ -6069,9 +6285,13 @@
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
     </row>
-    <row r="31" spans="1:25" ht="12.75">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
+    <row r="31" spans="1:25" ht="15">
+      <c r="A31" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
@@ -6096,9 +6316,13 @@
       <c r="X31" s="3"/>
       <c r="Y31" s="3"/>
     </row>
-    <row r="32" spans="1:25" ht="12.75">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
+    <row r="32" spans="1:25">
+      <c r="A32" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
@@ -6123,9 +6347,13 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
     </row>
-    <row r="33" spans="1:25" ht="12.75">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
+    <row r="33" spans="1:25" ht="47.25">
+      <c r="A33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
@@ -6150,9 +6378,13 @@
       <c r="X33" s="3"/>
       <c r="Y33" s="3"/>
     </row>
-    <row r="34" spans="1:25" ht="12.75">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
+    <row r="34" spans="1:25">
+      <c r="A34" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
@@ -6177,9 +6409,13 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
     </row>
-    <row r="35" spans="1:25" ht="12.75">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
+    <row r="35" spans="1:25" ht="45">
+      <c r="A35" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
@@ -6204,9 +6440,13 @@
       <c r="X35" s="3"/>
       <c r="Y35" s="3"/>
     </row>
-    <row r="36" spans="1:25" ht="12.75">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
+    <row r="36" spans="1:25" ht="31.5">
+      <c r="A36" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
@@ -6231,9 +6471,13 @@
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
     </row>
-    <row r="37" spans="1:25" ht="12.75">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
+    <row r="37" spans="1:25" ht="15">
+      <c r="A37" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
@@ -6258,9 +6502,13 @@
       <c r="X37" s="3"/>
       <c r="Y37" s="3"/>
     </row>
-    <row r="38" spans="1:25" ht="12.75">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
+    <row r="38" spans="1:25">
+      <c r="A38" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>97</v>
+      </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -6285,9 +6533,13 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
     </row>
-    <row r="39" spans="1:25" ht="12.75">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
+    <row r="39" spans="1:25" ht="47.25">
+      <c r="A39" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="22" t="s">
+        <v>96</v>
+      </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
@@ -6312,9 +6564,13 @@
       <c r="X39" s="3"/>
       <c r="Y39" s="3"/>
     </row>
-    <row r="40" spans="1:25" ht="12.75">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
+    <row r="40" spans="1:25">
+      <c r="A40" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
@@ -6339,9 +6595,13 @@
       <c r="X40" s="3"/>
       <c r="Y40" s="3"/>
     </row>
-    <row r="41" spans="1:25" ht="12.75">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
+    <row r="41" spans="1:25" ht="30">
+      <c r="A41" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>98</v>
+      </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
@@ -6366,9 +6626,13 @@
       <c r="X41" s="3"/>
       <c r="Y41" s="3"/>
     </row>
-    <row r="42" spans="1:25" ht="12.75">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
+    <row r="42" spans="1:25" ht="45">
+      <c r="A42" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" s="22" t="s">
+        <v>99</v>
+      </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
@@ -6393,9 +6657,13 @@
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
     </row>
-    <row r="43" spans="1:25" ht="12.75">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
+    <row r="43" spans="1:25" ht="15">
+      <c r="A43" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="24" t="s">
+        <v>59</v>
+      </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
@@ -6420,9 +6688,13 @@
       <c r="X43" s="3"/>
       <c r="Y43" s="3"/>
     </row>
-    <row r="44" spans="1:25" ht="12.75">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
+    <row r="44" spans="1:25">
+      <c r="A44" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>103</v>
+      </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -6447,9 +6719,13 @@
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
     </row>
-    <row r="45" spans="1:25" ht="12.75">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
+    <row r="45" spans="1:25" ht="47.25">
+      <c r="A45" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="22" t="s">
+        <v>100</v>
+      </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
@@ -6474,9 +6750,13 @@
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
     </row>
-    <row r="46" spans="1:25" ht="12.75">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
+    <row r="46" spans="1:25">
+      <c r="A46" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
@@ -6501,9 +6781,13 @@
       <c r="X46" s="3"/>
       <c r="Y46" s="3"/>
     </row>
-    <row r="47" spans="1:25" ht="12.75">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
+    <row r="47" spans="1:25" ht="60">
+      <c r="A47" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B47" s="22" t="s">
+        <v>101</v>
+      </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
@@ -6528,9 +6812,13 @@
       <c r="X47" s="3"/>
       <c r="Y47" s="3"/>
     </row>
-    <row r="48" spans="1:25" ht="12.75">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
+    <row r="48" spans="1:25" ht="31.5">
+      <c r="A48" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B48" s="22" t="s">
+        <v>102</v>
+      </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
@@ -6555,9 +6843,13 @@
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
     </row>
-    <row r="49" spans="1:25" ht="12.75">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
+    <row r="49" spans="1:25" ht="15">
+      <c r="A49" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="24" t="s">
+        <v>59</v>
+      </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
@@ -6582,9 +6874,13 @@
       <c r="X49" s="3"/>
       <c r="Y49" s="3"/>
     </row>
-    <row r="50" spans="1:25" ht="12.75">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
+    <row r="50" spans="1:25">
+      <c r="A50" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>104</v>
+      </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
@@ -6609,9 +6905,13 @@
       <c r="X50" s="3"/>
       <c r="Y50" s="3"/>
     </row>
-    <row r="51" spans="1:25" ht="12.75">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
+    <row r="51" spans="1:25" ht="47.25">
+      <c r="A51" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="22" t="s">
+        <v>105</v>
+      </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -6636,9 +6936,13 @@
       <c r="X51" s="3"/>
       <c r="Y51" s="3"/>
     </row>
-    <row r="52" spans="1:25" ht="12.75">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
+    <row r="52" spans="1:25">
+      <c r="A52" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="22" t="s">
+        <v>93</v>
+      </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
@@ -6663,9 +6967,13 @@
       <c r="X52" s="3"/>
       <c r="Y52" s="3"/>
     </row>
-    <row r="53" spans="1:25" ht="12.75">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
+    <row r="53" spans="1:25" ht="45">
+      <c r="A53" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="22" t="s">
+        <v>106</v>
+      </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -6690,9 +6998,13 @@
       <c r="X53" s="3"/>
       <c r="Y53" s="3"/>
     </row>
-    <row r="54" spans="1:25" ht="12.75">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
+    <row r="54" spans="1:25" ht="31.5">
+      <c r="A54" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" s="22" t="s">
+        <v>107</v>
+      </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
@@ -6718,8 +7030,6 @@
       <c r="Y54" s="3"/>
     </row>
     <row r="55" spans="1:25" ht="12.75">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
@@ -32313,6 +32623,168 @@
       <c r="X1002" s="3"/>
       <c r="Y1002" s="3"/>
     </row>
+    <row r="1003" spans="1:25" ht="12.75">
+      <c r="A1003" s="3"/>
+      <c r="B1003" s="3"/>
+      <c r="C1003" s="3"/>
+      <c r="D1003" s="3"/>
+      <c r="E1003" s="3"/>
+      <c r="F1003" s="3"/>
+      <c r="G1003" s="3"/>
+      <c r="H1003" s="3"/>
+      <c r="I1003" s="3"/>
+      <c r="J1003" s="3"/>
+      <c r="K1003" s="3"/>
+      <c r="L1003" s="3"/>
+      <c r="M1003" s="3"/>
+      <c r="N1003" s="3"/>
+      <c r="O1003" s="3"/>
+      <c r="P1003" s="3"/>
+      <c r="Q1003" s="3"/>
+      <c r="R1003" s="3"/>
+      <c r="S1003" s="3"/>
+      <c r="T1003" s="3"/>
+      <c r="U1003" s="3"/>
+      <c r="V1003" s="3"/>
+      <c r="W1003" s="3"/>
+      <c r="X1003" s="3"/>
+      <c r="Y1003" s="3"/>
+    </row>
+    <row r="1004" spans="1:25" ht="12.75">
+      <c r="A1004" s="3"/>
+      <c r="B1004" s="3"/>
+      <c r="C1004" s="3"/>
+      <c r="D1004" s="3"/>
+      <c r="E1004" s="3"/>
+      <c r="F1004" s="3"/>
+      <c r="G1004" s="3"/>
+      <c r="H1004" s="3"/>
+      <c r="I1004" s="3"/>
+      <c r="J1004" s="3"/>
+      <c r="K1004" s="3"/>
+      <c r="L1004" s="3"/>
+      <c r="M1004" s="3"/>
+      <c r="N1004" s="3"/>
+      <c r="O1004" s="3"/>
+      <c r="P1004" s="3"/>
+      <c r="Q1004" s="3"/>
+      <c r="R1004" s="3"/>
+      <c r="S1004" s="3"/>
+      <c r="T1004" s="3"/>
+      <c r="U1004" s="3"/>
+      <c r="V1004" s="3"/>
+      <c r="W1004" s="3"/>
+      <c r="X1004" s="3"/>
+      <c r="Y1004" s="3"/>
+    </row>
+    <row r="1005" spans="1:25" ht="12.75">
+      <c r="A1005" s="3"/>
+      <c r="B1005" s="3"/>
+      <c r="C1005" s="3"/>
+      <c r="D1005" s="3"/>
+      <c r="E1005" s="3"/>
+      <c r="F1005" s="3"/>
+      <c r="G1005" s="3"/>
+      <c r="H1005" s="3"/>
+      <c r="I1005" s="3"/>
+      <c r="J1005" s="3"/>
+      <c r="K1005" s="3"/>
+      <c r="L1005" s="3"/>
+      <c r="M1005" s="3"/>
+      <c r="N1005" s="3"/>
+      <c r="O1005" s="3"/>
+      <c r="P1005" s="3"/>
+      <c r="Q1005" s="3"/>
+      <c r="R1005" s="3"/>
+      <c r="S1005" s="3"/>
+      <c r="T1005" s="3"/>
+      <c r="U1005" s="3"/>
+      <c r="V1005" s="3"/>
+      <c r="W1005" s="3"/>
+      <c r="X1005" s="3"/>
+      <c r="Y1005" s="3"/>
+    </row>
+    <row r="1006" spans="1:25" ht="12.75">
+      <c r="A1006" s="3"/>
+      <c r="B1006" s="3"/>
+      <c r="C1006" s="3"/>
+      <c r="D1006" s="3"/>
+      <c r="E1006" s="3"/>
+      <c r="F1006" s="3"/>
+      <c r="G1006" s="3"/>
+      <c r="H1006" s="3"/>
+      <c r="I1006" s="3"/>
+      <c r="J1006" s="3"/>
+      <c r="K1006" s="3"/>
+      <c r="L1006" s="3"/>
+      <c r="M1006" s="3"/>
+      <c r="N1006" s="3"/>
+      <c r="O1006" s="3"/>
+      <c r="P1006" s="3"/>
+      <c r="Q1006" s="3"/>
+      <c r="R1006" s="3"/>
+      <c r="S1006" s="3"/>
+      <c r="T1006" s="3"/>
+      <c r="U1006" s="3"/>
+      <c r="V1006" s="3"/>
+      <c r="W1006" s="3"/>
+      <c r="X1006" s="3"/>
+      <c r="Y1006" s="3"/>
+    </row>
+    <row r="1007" spans="1:25" ht="12.75">
+      <c r="A1007" s="3"/>
+      <c r="B1007" s="3"/>
+      <c r="C1007" s="3"/>
+      <c r="D1007" s="3"/>
+      <c r="E1007" s="3"/>
+      <c r="F1007" s="3"/>
+      <c r="G1007" s="3"/>
+      <c r="H1007" s="3"/>
+      <c r="I1007" s="3"/>
+      <c r="J1007" s="3"/>
+      <c r="K1007" s="3"/>
+      <c r="L1007" s="3"/>
+      <c r="M1007" s="3"/>
+      <c r="N1007" s="3"/>
+      <c r="O1007" s="3"/>
+      <c r="P1007" s="3"/>
+      <c r="Q1007" s="3"/>
+      <c r="R1007" s="3"/>
+      <c r="S1007" s="3"/>
+      <c r="T1007" s="3"/>
+      <c r="U1007" s="3"/>
+      <c r="V1007" s="3"/>
+      <c r="W1007" s="3"/>
+      <c r="X1007" s="3"/>
+      <c r="Y1007" s="3"/>
+    </row>
+    <row r="1008" spans="1:25" ht="12.75">
+      <c r="A1008" s="3"/>
+      <c r="B1008" s="3"/>
+      <c r="C1008" s="3"/>
+      <c r="D1008" s="3"/>
+      <c r="E1008" s="3"/>
+      <c r="F1008" s="3"/>
+      <c r="G1008" s="3"/>
+      <c r="H1008" s="3"/>
+      <c r="I1008" s="3"/>
+      <c r="J1008" s="3"/>
+      <c r="K1008" s="3"/>
+      <c r="L1008" s="3"/>
+      <c r="M1008" s="3"/>
+      <c r="N1008" s="3"/>
+      <c r="O1008" s="3"/>
+      <c r="P1008" s="3"/>
+      <c r="Q1008" s="3"/>
+      <c r="R1008" s="3"/>
+      <c r="S1008" s="3"/>
+      <c r="T1008" s="3"/>
+      <c r="U1008" s="3"/>
+      <c r="V1008" s="3"/>
+      <c r="W1008" s="3"/>
+      <c r="X1008" s="3"/>
+      <c r="Y1008" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32331,10 +32803,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>68</v>
+      <c r="A1" s="17" t="s">
+        <v>61</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="18"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -32421,7 +32893,7 @@
     </row>
     <row r="4" spans="1:25" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="3"/>
@@ -32450,7 +32922,7 @@
     </row>
     <row r="5" spans="1:25" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="3"/>
@@ -32479,7 +32951,7 @@
     </row>
     <row r="6" spans="1:25" ht="30" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="3"/>
@@ -32508,7 +32980,7 @@
     </row>
     <row r="7" spans="1:25" ht="30" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="3"/>

</xml_diff>